<commit_message>
chore(sync): regeneracao 2026-06-10 + retomada + move Rastreabilidade + registros de sessao
- Regeneracao mecanica via auto_update_claude_md.py (data 10/06, paths de sessao cloud, contagem regressiva de prescricao em 300+ arquivos de auditoria/status)
- .continue-here.md: registro da Sessao 1 de organizacao da raiz (concluida)
- Move "Rastreabilidade Forense Completa" da raiz para relatorios/ (completa Fase B)
- 3 registros de sessao novos em relatorios/sessoes/
- 2 pastas _OUT_sync_referencias de 23/04 arquivadas em _ARQUIVO/

Fora deste commit (aguardando confirmacao de envio a PRODAM / correcao de citacoes):
Dashboard_PRODAM_Relatorio_Quinzenal_2026-06-10.html e _ORGANIZADO_2026-06-10/

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/DOSSIES_MULTIFORMATO/ADAF/dossie.xlsx
+++ b/DOSSIES_MULTIFORMATO/ADAF/dossie.xlsx
@@ -577,7 +577,11 @@
           <t>data_prescricao_proxima</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2028-04-30</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>